<commit_message>
3nd Exc UPD +  Fix BS JS
</commit_message>
<xml_diff>
--- a/dsd_checks/dati.xlsx
+++ b/dsd_checks/dati.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\dsd_checks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6542611E-997E-4392-BBCF-F5CD6C5D634E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCD50841-A8BF-483D-9DD2-D2C6437A3546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="56">
   <si>
     <t>Data</t>
   </si>
@@ -183,14 +183,6 @@
     <t>19:01</t>
   </si>
   <si>
-    <t>Given yesterday's blood values, I wanted to do a little test today, and I tried eating other carbohydrates for lunch,
-eating 2 more toasts (whole wheat) with butter (obviously the light one I bought),
-so as to try to understand how my body would react (despite insulin and pills for the pancreas).
-I had to move the Lantax to a range that goes between 14:00 and 15:00
-because between 16:00 and 17:00 it becomes a problem for me to manage it,
-given that it is a time that does not match with my daily eating or general routine.</t>
-  </si>
-  <si>
     <t>For dinner, I did another test... &lt;br&gt;
 This time I made a mixed salad with: &lt;br&gt;
 - Tomatoes &lt;br&gt;
@@ -217,6 +209,26 @@
 Additionally, yesterday's test demonstrated the type of carbohydrate tolerance my body currently has (taking insulin),&lt;br&gt;
 and also the effectiveness of having a mixed protein salad for dinner which lowered my blood sugar by 2.8 overnight,&lt;br&gt;
 causing me to wake up with a blood sugar level that was lower than I've had in the previous 2 mornings.</t>
+  </si>
+  <si>
+    <t>14:00</t>
+  </si>
+  <si>
+    <t>I made a mixed salad with: &lt;br&gt;
+- Tomatoes &lt;br&gt;
+- Cucumbers &lt;br&gt;
+- Green Olives &lt;br&gt;
+- Basil &lt;br&gt;
+- Tuna &lt;br&gt;
+- 1 tablespoon Extra Virgin Olive Oil (EVO)&lt;br&gt;
+&lt;br&gt;
+It's the same salad as the other day but without the yogurt as dressing&lt;br&gt;
+because last time it made the salad have a sour aftertaste.</t>
+  </si>
+  <si>
+    <t>Given yesterday's blood values, I wanted to do a little test today, and I tried eating other carbohydrates for lunch,
+eating 2 more toasts (whole wheat) with butter (obviously the light one I bought),
+so as to try to understand how my body would react (despite insulin and pills for the pancreas).</t>
   </si>
 </sst>
 </file>
@@ -823,7 +835,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="210" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="105" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <f>A6</f>
         <v>46208</v>
@@ -846,7 +858,7 @@
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="13" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="I7" s="4">
         <v>28</v>
@@ -905,10 +917,10 @@
         <v>0</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H9" s="13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I9" s="4">
         <v>0</v>
@@ -930,7 +942,7 @@
         <v>10</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E10" s="4">
         <v>12.3</v>
@@ -940,7 +952,7 @@
       </c>
       <c r="G10" s="4"/>
       <c r="H10" s="13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I10" s="4">
         <v>0</v>
@@ -949,7 +961,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="180" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <f>A10</f>
         <v>46209</v>
@@ -961,13 +973,27 @@
       <c r="C11" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="10"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
+      <c r="D11" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E11" s="4">
+        <v>12.8</v>
+      </c>
+      <c r="F11" s="4">
+        <v>0</v>
+      </c>
+      <c r="G11" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="H11" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="I11" s="4">
+        <v>0</v>
+      </c>
+      <c r="J11" s="4">
+        <v>20</v>
+      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
@@ -981,13 +1007,25 @@
       <c r="C12" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D12" s="10"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
+      <c r="D12" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="E12" s="4">
+        <v>7.5</v>
+      </c>
+      <c r="F12" s="4">
+        <v>0</v>
+      </c>
       <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
+      <c r="H12" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I12" s="4">
+        <v>0</v>
+      </c>
+      <c r="J12" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
@@ -8030,6 +8068,7 @@
   <hyperlinks>
     <hyperlink ref="G5" r:id="rId1" xr:uid="{100DED73-170C-4584-AF8A-5BBE9938D1B2}"/>
     <hyperlink ref="G9" r:id="rId2" xr:uid="{BBEA467B-A84F-488C-97AE-7EA598984E70}"/>
+    <hyperlink ref="G11" r:id="rId3" xr:uid="{25B97C21-83A5-486E-A4EE-C8B043C82D3E}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
7th Exc UPD 2Days 2gether
</commit_message>
<xml_diff>
--- a/dsd_checks/dati.xlsx
+++ b/dsd_checks/dati.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\dsd_checks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DD38594-6159-483A-BDEE-6BBB238F9C7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0714ABE5-0645-421D-BDB3-C93009EFF491}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="78">
   <si>
     <t>Data</t>
   </si>
@@ -255,13 +255,6 @@
     <t>17:00</t>
   </si>
   <si>
-    <t>I didn't eat, just took LANTAX&lt;br&gt;
-&lt;br&gt;
-18:00 - UPDATE:&lt;br&gt;
-LANTAX dropped the BS from 15.4 to 11.3.&lt;br&gt;
-That is: 4.1 in just over 1 hour.</t>
-  </si>
-  <si>
     <t>21:30</t>
   </si>
   <si>
@@ -307,6 +300,47 @@
 &lt;br&gt;
 23:54 - UPDATE:&lt;br&gt;
 BS dropped 6,7&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>13:46</t>
+  </si>
+  <si>
+    <t>I didn't eat, just took LANTUS&lt;br&gt;
+&lt;br&gt;
+18:00 - UPDATE:&lt;br&gt;
+LANTUS dropped the BS from 15.4 to 11.3.&lt;br&gt;
+That is: 4.1 in just over 1 hour.</t>
+  </si>
+  <si>
+    <t>LANTUS</t>
+  </si>
+  <si>
+    <t>Pasta Amatriciana:&lt;br&gt;
+- Pasta - Whole Wheat Spaghetti&lt;br&gt;
+- Tomato Sauce&lt;br&gt;
+- Bacon&lt;br&gt;
+- Parmesan Cheese&lt;br&gt;
+- Chipotle Pepper</t>
+  </si>
+  <si>
+    <t>Yogurt with 1 Tesco Wheat Biscuits&lt;br&gt;
+and Black Coffee with some skimmed milk</t>
+  </si>
+  <si>
+    <t>Mixed salad with:&lt;br&gt;
+- Tomatoes&lt;br&gt;
+- Cucumbers&lt;br&gt;
+- Green Olives&lt;br&gt;
+- Tuna&lt;br&gt;
+- 2 tablespoons Extra Virgin Olive Oil (EVO)</t>
+  </si>
+  <si>
+    <t>mixed salad with:&lt;br&gt;
+- Tomatoes&lt;br&gt;
+- Cucumbers&lt;br&gt;
+- Green Olives&lt;br&gt;
+- Tuna&lt;br&gt;
+- 2 tablespoons Extra Virgin Olive Oil (EVO)</t>
   </si>
 </sst>
 </file>
@@ -1227,7 +1261,7 @@
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="13" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="I16" s="4">
         <v>30</v>
@@ -1249,7 +1283,7 @@
         <v>13</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E17" s="4">
         <v>9.6999999999999993</v>
@@ -1258,10 +1292,10 @@
         <v>0</v>
       </c>
       <c r="G17" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="H17" s="13" t="s">
         <v>64</v>
-      </c>
-      <c r="H17" s="13" t="s">
-        <v>65</v>
       </c>
       <c r="I17" s="4"/>
       <c r="J17" s="4">
@@ -1281,7 +1315,7 @@
         <v>10</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E18" s="4">
         <v>12.6</v>
@@ -1291,7 +1325,7 @@
       </c>
       <c r="G18" s="4"/>
       <c r="H18" s="13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I18" s="4">
         <v>0</v>
@@ -1322,10 +1356,10 @@
         <v>0.1</v>
       </c>
       <c r="G19" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="H19" s="13" t="s">
         <v>68</v>
-      </c>
-      <c r="H19" s="13" t="s">
-        <v>69</v>
       </c>
       <c r="I19" s="4">
         <v>30</v>
@@ -1347,7 +1381,7 @@
         <v>12</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E20" s="4">
         <v>11.7</v>
@@ -1379,7 +1413,7 @@
         <v>13</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E21" s="4">
         <v>10.8</v>
@@ -1389,7 +1423,7 @@
       </c>
       <c r="G21" s="4"/>
       <c r="H21" s="13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I21" s="4">
         <v>0</v>
@@ -1418,7 +1452,7 @@
       <c r="I22" s="4"/>
       <c r="J22" s="4"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" ht="90" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <f>A22</f>
         <v>46212</v>
@@ -1430,13 +1464,25 @@
       <c r="C23" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D23" s="10"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
+      <c r="D23" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="E23" s="4">
+        <v>15.4</v>
+      </c>
+      <c r="F23" s="4">
+        <v>0.1</v>
+      </c>
       <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
-      <c r="I23" s="4"/>
-      <c r="J23" s="4"/>
+      <c r="H23" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="I23" s="4">
+        <v>0</v>
+      </c>
+      <c r="J23" s="4">
+        <v>20</v>
+      </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
@@ -1450,15 +1496,27 @@
       <c r="C24" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D24" s="10"/>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
+      <c r="D24" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="E24" s="4">
+        <v>9.1999999999999993</v>
+      </c>
+      <c r="F24" s="4">
+        <v>0</v>
+      </c>
       <c r="G24" s="4"/>
-      <c r="H24" s="4"/>
-      <c r="I24" s="4"/>
-      <c r="J24" s="4"/>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H24" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="I24" s="4">
+        <v>30</v>
+      </c>
+      <c r="J24" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="90" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <f>A24</f>
         <v>46212</v>
@@ -1470,15 +1528,27 @@
       <c r="C25" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D25" s="10"/>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
+      <c r="D25" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="E25" s="4">
+        <v>7.5</v>
+      </c>
+      <c r="F25" s="4">
+        <v>0</v>
+      </c>
       <c r="G25" s="4"/>
-      <c r="H25" s="4"/>
-      <c r="I25" s="4"/>
-      <c r="J25" s="4"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H25" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="I25" s="4">
+        <v>0</v>
+      </c>
+      <c r="J25" s="4">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <f>A22+1</f>
         <v>46213</v>
@@ -1490,15 +1560,27 @@
       <c r="C26" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D26" s="10"/>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
+      <c r="D26" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="E26" s="4">
+        <v>17.7</v>
+      </c>
+      <c r="F26" s="4">
+        <v>0.1</v>
+      </c>
       <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="4"/>
-      <c r="J26" s="4"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H26" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="I26" s="4">
+        <v>0</v>
+      </c>
+      <c r="J26" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="90" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <f>A26</f>
         <v>46213</v>
@@ -1510,13 +1592,25 @@
       <c r="C27" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D27" s="10"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
+      <c r="D27" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="E27" s="4">
+        <v>6.1</v>
+      </c>
+      <c r="F27" s="4">
+        <v>0</v>
+      </c>
       <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
-      <c r="I27" s="4"/>
-      <c r="J27" s="4"/>
+      <c r="H27" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="I27" s="4">
+        <v>0</v>
+      </c>
+      <c r="J27" s="4">
+        <v>15</v>
+      </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="2">

</xml_diff>